<commit_message>
best run 200126 216pm
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_mexico_transformation_strategy_pemex.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_mexico_transformation_strategy_pemex.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_mexico/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD0123B7-A1C1-604C-9C4D-EBCF745836E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F692A54B-84A8-144C-AC4C-7B8056F7347B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-40380" yWindow="-7160" windowWidth="35300" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -2010,10 +2010,12 @@
         <v>0.45</v>
       </c>
       <c r="L2" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
+      <c r="N2" s="13">
+        <v>3</v>
+      </c>
       <c r="O2" s="13"/>
       <c r="P2" s="13"/>
       <c r="Q2" s="13"/>
@@ -2045,10 +2047,12 @@
         <v>0.5</v>
       </c>
       <c r="L3" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
+      <c r="N3" s="13">
+        <v>3</v>
+      </c>
       <c r="O3" s="13"/>
       <c r="P3" s="13"/>
       <c r="Q3" s="13"/>
@@ -2080,10 +2084,12 @@
         <v>0.3</v>
       </c>
       <c r="L4" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
+      <c r="N4" s="13">
+        <v>3</v>
+      </c>
       <c r="O4" s="13"/>
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
@@ -2115,10 +2121,12 @@
         <v>217</v>
       </c>
       <c r="L5" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
+      <c r="N5" s="13">
+        <v>1</v>
+      </c>
       <c r="O5" s="13"/>
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
@@ -2154,7 +2162,7 @@
         <v>0.2</v>
       </c>
       <c r="L6" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M6" s="13"/>
       <c r="N6" s="13"/>
@@ -2189,7 +2197,7 @@
         <v>50</v>
       </c>
       <c r="L7" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M7" s="13"/>
       <c r="N7" s="13"/>
@@ -2228,7 +2236,7 @@
         <v>229</v>
       </c>
       <c r="L8" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
@@ -2267,7 +2275,7 @@
         <v>0.95</v>
       </c>
       <c r="L9" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
@@ -2306,11 +2314,11 @@
         <v>0.95</v>
       </c>
       <c r="L10" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M10" s="13"/>
       <c r="N10" s="13">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="O10" s="13"/>
       <c r="P10" s="13"/>
@@ -2343,7 +2351,7 @@
         <v>0.8</v>
       </c>
       <c r="L11" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M11" s="13"/>
       <c r="N11" s="13"/>
@@ -2378,7 +2386,7 @@
         <v>0.8</v>
       </c>
       <c r="L12" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M12" s="13"/>
       <c r="N12" s="13"/>
@@ -2417,7 +2425,7 @@
         <v>0.3</v>
       </c>
       <c r="L13" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
@@ -2456,7 +2464,7 @@
         <v>0.4</v>
       </c>
       <c r="L14" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="13"/>
@@ -2491,10 +2499,12 @@
         <v>252</v>
       </c>
       <c r="L15" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M15" s="13"/>
-      <c r="N15" s="13"/>
+      <c r="N15" s="13">
+        <v>1</v>
+      </c>
       <c r="O15" s="13"/>
       <c r="P15" s="13"/>
       <c r="Q15" s="13"/>
@@ -2530,7 +2540,7 @@
         <v>0.5</v>
       </c>
       <c r="L16" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="13">
@@ -2571,7 +2581,7 @@
         <v>0.3</v>
       </c>
       <c r="L17" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="13">
@@ -2612,10 +2622,12 @@
         <v>0.1</v>
       </c>
       <c r="L18" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M18" s="13"/>
-      <c r="N18" s="13"/>
+      <c r="N18" s="13">
+        <v>1</v>
+      </c>
       <c r="O18" s="13"/>
       <c r="P18" s="13"/>
       <c r="Q18" s="13"/>
@@ -2647,10 +2659,12 @@
         <v>0.1</v>
       </c>
       <c r="L19" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M19" s="13"/>
-      <c r="N19" s="13"/>
+      <c r="N19" s="13">
+        <v>1</v>
+      </c>
       <c r="O19" s="13"/>
       <c r="P19" s="13"/>
       <c r="Q19" s="13"/>
@@ -2682,10 +2696,12 @@
         <v>0.1</v>
       </c>
       <c r="L20" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M20" s="13"/>
-      <c r="N20" s="13"/>
+      <c r="N20" s="13">
+        <v>1</v>
+      </c>
       <c r="O20" s="13"/>
       <c r="P20" s="13"/>
       <c r="Q20" s="13"/>
@@ -2717,10 +2733,12 @@
         <v>0.1</v>
       </c>
       <c r="L21" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M21" s="13"/>
-      <c r="N21" s="13"/>
+      <c r="N21" s="13">
+        <v>1</v>
+      </c>
       <c r="O21" s="13"/>
       <c r="P21" s="13"/>
       <c r="Q21" s="13"/>
@@ -2756,7 +2774,7 @@
         <v>0.999</v>
       </c>
       <c r="L22" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M22" s="13"/>
       <c r="N22" s="13"/>
@@ -2795,7 +2813,7 @@
         <v>0.95</v>
       </c>
       <c r="L23" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M23" s="13"/>
       <c r="N23" s="13"/>
@@ -2834,7 +2852,7 @@
         <v>0.2</v>
       </c>
       <c r="L24" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
@@ -2873,7 +2891,7 @@
         <v>0.1</v>
       </c>
       <c r="L25" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
@@ -2908,7 +2926,7 @@
         <v>0.9</v>
       </c>
       <c r="L26" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
@@ -2943,7 +2961,7 @@
         <v>291</v>
       </c>
       <c r="L27" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
@@ -2978,7 +2996,7 @@
         <v>293</v>
       </c>
       <c r="L28" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
@@ -3013,7 +3031,7 @@
         <v>295</v>
       </c>
       <c r="L29" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M29" s="13"/>
       <c r="N29" s="13"/>
@@ -3048,7 +3066,7 @@
         <v>298</v>
       </c>
       <c r="L30" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M30" s="13"/>
       <c r="N30" s="13"/>
@@ -3083,7 +3101,7 @@
         <v>0.5</v>
       </c>
       <c r="L31" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M31" s="13"/>
       <c r="N31" s="13"/>
@@ -3122,7 +3140,7 @@
         <v>0.3</v>
       </c>
       <c r="L32" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M32" s="13"/>
       <c r="N32" s="13"/>
@@ -3157,7 +3175,7 @@
         <v>0.5</v>
       </c>
       <c r="L33" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M33" s="13"/>
       <c r="N33" s="13"/>
@@ -3192,7 +3210,7 @@
         <v>0.9</v>
       </c>
       <c r="L34" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M34" s="13"/>
       <c r="N34" s="13"/>
@@ -3227,7 +3245,7 @@
         <v>0.5</v>
       </c>
       <c r="L35" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M35" s="13"/>
       <c r="N35" s="13"/>
@@ -3262,7 +3280,7 @@
         <v>0.5</v>
       </c>
       <c r="L36" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M36" s="13"/>
       <c r="N36" s="13"/>
@@ -3297,7 +3315,7 @@
         <v>0.95</v>
       </c>
       <c r="L37" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M37" s="13"/>
       <c r="N37" s="13"/>
@@ -3332,7 +3350,7 @@
         <v>0.2</v>
       </c>
       <c r="L38" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M38" s="13"/>
       <c r="N38" s="13"/>
@@ -3367,7 +3385,7 @@
         <v>0.2</v>
       </c>
       <c r="L39" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M39" s="13"/>
       <c r="N39" s="13"/>
@@ -3406,10 +3424,10 @@
         <v>0.25</v>
       </c>
       <c r="L40" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M40" s="13">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="N40" s="13">
         <v>2</v>
@@ -3449,13 +3467,13 @@
         <v>0.25</v>
       </c>
       <c r="L41" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M41" s="13">
         <v>1</v>
       </c>
       <c r="N41" s="13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O41" s="13"/>
       <c r="P41" s="13"/>
@@ -3492,12 +3510,10 @@
         <v>0.25</v>
       </c>
       <c r="L42" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M42" s="13"/>
-      <c r="N42" s="13">
-        <v>2</v>
-      </c>
+      <c r="N42" s="13"/>
       <c r="O42" s="13"/>
       <c r="P42" s="13"/>
       <c r="Q42" s="13"/>
@@ -3529,7 +3545,7 @@
         <v>0.25</v>
       </c>
       <c r="L43" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M43" s="13"/>
       <c r="N43" s="13">
@@ -3566,10 +3582,12 @@
         <v>0.7</v>
       </c>
       <c r="L44" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M44" s="13"/>
-      <c r="N44" s="13"/>
+      <c r="N44" s="13">
+        <v>1</v>
+      </c>
       <c r="O44" s="13"/>
       <c r="P44" s="13"/>
       <c r="Q44" s="13"/>
@@ -3605,7 +3623,7 @@
         <v>0.7</v>
       </c>
       <c r="L45" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M45" s="13"/>
       <c r="N45" s="13">
@@ -3646,10 +3664,12 @@
         <v>0.7</v>
       </c>
       <c r="L46" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M46" s="13"/>
-      <c r="N46" s="13"/>
+      <c r="N46" s="13">
+        <v>1</v>
+      </c>
       <c r="O46" s="13"/>
       <c r="P46" s="13"/>
       <c r="Q46" s="13"/>
@@ -3681,10 +3701,12 @@
         <v>0.25</v>
       </c>
       <c r="L47" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M47" s="13"/>
-      <c r="N47" s="13"/>
+      <c r="N47" s="13">
+        <v>1</v>
+      </c>
       <c r="O47" s="13"/>
       <c r="P47" s="13"/>
       <c r="Q47" s="13"/>
@@ -3720,7 +3742,7 @@
         <v>0.2</v>
       </c>
       <c r="L48" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M48" s="13"/>
       <c r="N48" s="13">
@@ -3761,7 +3783,7 @@
         <v>0.3</v>
       </c>
       <c r="L49" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M49" s="13"/>
       <c r="N49" s="13">
@@ -3802,10 +3824,12 @@
         <v>358</v>
       </c>
       <c r="L50" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M50" s="13"/>
-      <c r="N50" s="13"/>
+      <c r="N50" s="13">
+        <v>1</v>
+      </c>
       <c r="O50" s="13"/>
       <c r="P50" s="13"/>
       <c r="Q50" s="13"/>
@@ -3837,7 +3861,7 @@
         <v>0.85</v>
       </c>
       <c r="L51" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M51" s="13"/>
       <c r="N51" s="13"/>
@@ -3876,7 +3900,7 @@
         <v>0.9</v>
       </c>
       <c r="L52" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M52" s="13"/>
       <c r="N52" s="13"/>
@@ -3915,10 +3939,12 @@
         <v>370</v>
       </c>
       <c r="L53" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M53" s="13"/>
-      <c r="N53" s="13"/>
+      <c r="N53" s="13">
+        <v>1</v>
+      </c>
       <c r="O53" s="13"/>
       <c r="P53" s="13"/>
       <c r="Q53" s="13"/>
@@ -3954,7 +3980,7 @@
         <v>374</v>
       </c>
       <c r="L54" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M54" s="13"/>
       <c r="N54" s="13"/>
@@ -3993,7 +4019,7 @@
         <v>378</v>
       </c>
       <c r="L55" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M55" s="13"/>
       <c r="N55" s="13"/>
@@ -4032,10 +4058,12 @@
         <v>0.3</v>
       </c>
       <c r="L56" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M56" s="13"/>
-      <c r="N56" s="13"/>
+      <c r="N56" s="13">
+        <v>1</v>
+      </c>
       <c r="O56" s="13"/>
       <c r="P56" s="13"/>
       <c r="Q56" s="13"/>
@@ -4067,10 +4095,12 @@
         <v>385</v>
       </c>
       <c r="L57" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M57" s="13"/>
-      <c r="N57" s="13"/>
+      <c r="N57" s="13">
+        <v>1</v>
+      </c>
       <c r="O57" s="13"/>
       <c r="P57" s="13"/>
       <c r="Q57" s="13"/>
@@ -4106,7 +4136,7 @@
         <v>0.85</v>
       </c>
       <c r="L58" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M58" s="13"/>
       <c r="N58" s="13"/>
@@ -4141,7 +4171,7 @@
         <v>0.85</v>
       </c>
       <c r="L59" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M59" s="13"/>
       <c r="N59" s="13"/>
@@ -4176,10 +4206,12 @@
         <v>0.85</v>
       </c>
       <c r="L60" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M60" s="13"/>
-      <c r="N60" s="13"/>
+      <c r="N60" s="13">
+        <v>1</v>
+      </c>
       <c r="O60" s="13"/>
       <c r="P60" s="13"/>
       <c r="Q60" s="13"/>
@@ -4215,7 +4247,7 @@
         <v>1</v>
       </c>
       <c r="L61" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M61" s="13"/>
       <c r="N61" s="13"/>
@@ -4254,10 +4286,12 @@
         <v>0.95</v>
       </c>
       <c r="L62" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M62" s="13"/>
-      <c r="N62" s="13"/>
+      <c r="N62" s="13">
+        <v>1</v>
+      </c>
       <c r="O62" s="13"/>
       <c r="P62" s="13"/>
       <c r="Q62" s="13"/>
@@ -4291,7 +4325,7 @@
         <v>0.8</v>
       </c>
       <c r="L63" s="10">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M63" s="13"/>
       <c r="N63" s="13"/>
@@ -4418,8 +4452,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N39 N51:N62">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="N40">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4430,8 +4464,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N40">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="N41:N50">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N51:N62 N2:N39">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4526,18 +4572,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N41:N50">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
update natural gas prices
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_mexico_transformation_strategy_pemex.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_mexico_transformation_strategy_pemex.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabianfuentes/git/ssp_mexico/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C00AF6-4A4E-814F-B7A3-02C9AB5DAF59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D52EE6C-542C-7945-8ED4-A65D446392FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="-7160" windowWidth="25600" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-40660" yWindow="-7160" windowWidth="30540" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="418">
   <si>
     <t>subsector</t>
   </si>
@@ -1329,6 +1329,15 @@
   </si>
   <si>
     <t>strategy_5</t>
+  </si>
+  <si>
+    <t>TX:ENFU:ADJ_PRICES</t>
+  </si>
+  <si>
+    <t>Increase OR Decrease prices of fuels</t>
+  </si>
+  <si>
+    <t>transformation_enfu_adj_prices.yaml</t>
   </si>
 </sst>
 </file>
@@ -4792,24 +4801,44 @@
       </c>
       <c r="R63" s="42"/>
     </row>
-    <row r="64" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="16"/>
-      <c r="B64" s="16"/>
-      <c r="C64" s="16"/>
-      <c r="D64" s="16"/>
-      <c r="E64" s="16"/>
-      <c r="F64" s="16"/>
-      <c r="G64" s="16"/>
-      <c r="H64" s="16"/>
-      <c r="I64" s="16"/>
-      <c r="J64" s="16"/>
-      <c r="K64" s="29"/>
-      <c r="L64" s="28"/>
-      <c r="M64" s="25"/>
-      <c r="N64" s="25"/>
-      <c r="O64" s="25"/>
-      <c r="P64" s="25"/>
-      <c r="Q64" s="25"/>
+    <row r="64" spans="1:18" ht="52" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="B64" s="23" t="s">
+        <v>407</v>
+      </c>
+      <c r="C64" s="39" t="s">
+        <v>415</v>
+      </c>
+      <c r="D64" s="36"/>
+      <c r="E64" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="F64" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="G64" s="9"/>
+      <c r="H64" s="9"/>
+      <c r="I64" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="J64" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="K64" s="15">
+        <v>0.8</v>
+      </c>
+      <c r="L64" s="10">
+        <v>10</v>
+      </c>
+      <c r="M64" s="13"/>
+      <c r="N64" s="13"/>
+      <c r="O64" s="13"/>
+      <c r="P64" s="13"/>
+      <c r="Q64" s="13">
+        <v>1</v>
+      </c>
     </row>
     <row r="65" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="16"/>
@@ -4880,7 +4909,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M64:M1048576 M1:M7 M47:M62 M9:M12 M14 M63:Q63 M16:M45">
+  <conditionalFormatting sqref="M65:M1048576 M1:M7 M47:M62 M9:M12 M14 M16:M45 M63:Q64">
     <cfRule type="colorScale" priority="46">
       <colorScale>
         <cfvo type="min"/>
@@ -4892,7 +4921,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N64:N1048576">
+  <conditionalFormatting sqref="N65:N1048576">
     <cfRule type="colorScale" priority="58">
       <colorScale>
         <cfvo type="min"/>
@@ -4928,7 +4957,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O64:O1048576">
+  <conditionalFormatting sqref="O65:O1048576">
     <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
@@ -4940,7 +4969,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P64:P1048576">
+  <conditionalFormatting sqref="P65:P1048576">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
@@ -4964,7 +4993,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q64:Q1048576">
+  <conditionalFormatting sqref="Q65:Q1048576">
     <cfRule type="colorScale" priority="53">
       <colorScale>
         <cfvo type="min"/>
@@ -4985,7 +5014,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5" style="3" bestFit="1" customWidth="1"/>
@@ -5876,6 +5905,20 @@
         <v>409</v>
       </c>
     </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>417</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>